<commit_message>
bob file for plc
</commit_message>
<xml_diff>
--- a/ioc/rfTestStandApp/Db/PLC_Tags.xlsx
+++ b/ioc/rfTestStandApp/Db/PLC_Tags.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/1h7/projects/mpex-rf-test-stand/epics/ioc/rfTestStandApp/Db/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E207FF40-BA1D-E542-A6BE-E399D691F3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC30677-B54C-424A-9739-8A004811BAD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2200" yWindow="600" windowWidth="77800" windowHeight="26440" xr2:uid="{3FE3484D-6191-BF43-92D0-7162105C2A70}"/>
+    <workbookView xWindow="66200" yWindow="0" windowWidth="77800" windowHeight="26440" activeTab="1" xr2:uid="{3FE3484D-6191-BF43-92D0-7162105C2A70}"/>
   </bookViews>
   <sheets>
     <sheet name="example" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="104">
   <si>
     <t>recordType</t>
   </si>
@@ -346,6 +346,9 @@
   </si>
   <si>
     <t>$(S):Mot:ErrRst-Cmd</t>
+  </si>
+  <si>
+    <t>DRVL</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1175,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{837BD51E-EF3A-1E4D-9B13-DEAD21AFD473}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="15"/>
@@ -1191,7 +1194,7 @@
     <col min="14" max="16384" width="10.83203125" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -1234,8 +1237,11 @@
       <c r="N1" s="14" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="O1" s="19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="13"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -1250,7 +1256,7 @@
       <c r="L2" s="13"/>
       <c r="M2" s="14"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
         <v>18</v>
       </c>
@@ -1272,13 +1278,13 @@
       <c r="G3" s="16"/>
       <c r="M3" s="19"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
       <c r="D4" s="16"/>
       <c r="G4" s="16"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>12</v>
       </c>
@@ -1301,7 +1307,7 @@
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
         <v>12</v>
       </c>
@@ -1324,7 +1330,7 @@
       <c r="I6" s="19"/>
       <c r="J6" s="19"/>
     </row>
-    <row r="7" spans="1:14" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" s="17" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
         <v>12</v>
       </c>
@@ -1346,7 +1352,7 @@
       <c r="I7" s="20"/>
       <c r="J7" s="20"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
         <v>12</v>
       </c>
@@ -1369,7 +1375,7 @@
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>12</v>
       </c>
@@ -1392,13 +1398,13 @@
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="G10" s="16"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
         <v>54</v>
       </c>
@@ -1420,8 +1426,9 @@
       </c>
       <c r="M11" s="19"/>
       <c r="N11" s="19"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O11" s="19"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
         <v>54</v>
       </c>
@@ -1443,14 +1450,15 @@
       </c>
       <c r="M12" s="19"/>
       <c r="N12" s="19"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O12" s="19"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="15" t="s">
         <v>16</v>
       </c>
@@ -1473,7 +1481,7 @@
       <c r="I14" s="19"/>
       <c r="J14" s="19"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>16</v>
       </c>
@@ -1496,7 +1504,7 @@
       <c r="I15" s="19"/>
       <c r="J15" s="19"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="15" t="s">
         <v>16</v>
       </c>

</xml_diff>